<commit_message>
Add location/timing/campaign-id support to in-app message publishing
Adds CampaignId, Style (banner/modal/fullscreen), StartDate, and EndDate
columns to the InAppMessages sheet. Active is now computed from Active AND
the StartDate/EndDate window at publish time, and both dates are passed
through in the payload so the client can re-check the window between
publishes. README documents Remote Config's built-in Country/Region
condition for location targeting and walks through a location + modal +
timed + campaign-id example end to end.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RzBUj3Jg1FCpCQei32m38A
</commit_message>
<xml_diff>
--- a/firebase-campaign-tool/templates/campaign-template.xlsx
+++ b/firebase-campaign-tool/templates/campaign-template.xlsx
@@ -449,7 +449,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:L3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -474,6 +474,18 @@
         <v>Condition</v>
       </c>
       <c r="H1" t="str">
+        <v>CampaignId</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Style</v>
+      </c>
+      <c r="J1" t="str">
+        <v>StartDate</v>
+      </c>
+      <c r="K1" t="str">
+        <v>EndDate</v>
+      </c>
+      <c r="L1" t="str">
         <v>Active</v>
       </c>
     </row>
@@ -500,12 +512,62 @@
         <v/>
       </c>
       <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>banner</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v>TRUE</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>mumbai-store-launch</v>
+      </c>
+      <c r="B3" t="str">
+        <v>We just opened in Mumbai!</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Visit our new store and get 15% off your first purchase.</v>
+      </c>
+      <c r="D3" t="str">
+        <v>https://example.com/images/mumbai-launch.png</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Get Directions</v>
+      </c>
+      <c r="F3" t="str">
+        <v>https://example.com/stores/mumbai</v>
+      </c>
+      <c r="G3" t="str">
+        <v>India Users</v>
+      </c>
+      <c r="H3" t="str">
+        <v>mumbai-launch-2026</v>
+      </c>
+      <c r="I3" t="str">
+        <v>modal</v>
+      </c>
+      <c r="J3" t="str">
+        <v>2026-09-10T09:00:00Z</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2026-09-17T23:59:59Z</v>
+      </c>
+      <c r="L3" t="str">
         <v>TRUE</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>